<commit_message>
mise à jour du projet
</commit_message>
<xml_diff>
--- a/media/rapports/excel/facturation.xlsx
+++ b/media/rapports/excel/facturation.xlsx
@@ -424,18 +424,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -488,17 +488,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FN/53/2026</t>
+          <t>FN/52/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ndayishimiye emmanuel</t>
+          <t>ISM IRAKIZA SPARE MOTORS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -512,29 +512,29 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1000000</v>
+        <v>377966.12</v>
       </c>
       <c r="G2" t="n">
-        <v>180000</v>
+        <v>68033.89999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>1180000</v>
+        <v>446000.02</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ANNULE</t>
+          <t>ENVOYE</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FN/52/2026</t>
+          <t>FN/49/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -553,24 +553,24 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>377966.12</v>
+        <v>6779.68</v>
       </c>
       <c r="G3" t="n">
-        <v>68033.89999999999</v>
+        <v>1220.34</v>
       </c>
       <c r="H3" t="n">
-        <v>446000.02</v>
+        <v>8000.02</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ANNULE</t>
+          <t>ENVOYE</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FN/49/2026</t>
+          <t>FA/33/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>FN — Facture Normale</t>
+          <t>FA — Facture Avoir / Note de Crédit</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -594,13 +594,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>6779.68</v>
+        <v>3389.84</v>
       </c>
       <c r="G4" t="n">
-        <v>1220.34</v>
+        <v>610.17</v>
       </c>
       <c r="H4" t="n">
-        <v>8000.02</v>
+        <v>4000.01</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -611,7 +611,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FA/33/2026</t>
+          <t>FN/51/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -621,12 +621,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ISM IRAKIZA SPARE MOTORS</t>
+          <t>Ndayishimiye emmanuel</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>FA — Facture Avoir / Note de Crédit</t>
+          <t>FN — Facture Normale</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -635,13 +635,13 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3389.84</v>
+        <v>1182203.4</v>
       </c>
       <c r="G5" t="n">
-        <v>610.17</v>
+        <v>212796.61</v>
       </c>
       <c r="H5" t="n">
-        <v>4000.01</v>
+        <v>1395000.01</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -652,17 +652,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FN/51/2026</t>
+          <t>FN/44/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ndayishimiye emmanuel</t>
+          <t>ISM IRAKIZA SPARE MOTORS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -676,13 +676,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1182203.4</v>
+        <v>472881.36</v>
       </c>
       <c r="G6" t="n">
-        <v>212796.61</v>
+        <v>85118.64</v>
       </c>
       <c r="H6" t="n">
-        <v>1395000.01</v>
+        <v>558000</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -693,7 +693,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FN/44/2026</t>
+          <t>FA/31/2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>FN — Facture Normale</t>
+          <t>FA — Facture Avoir / Note de Crédit</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -717,13 +717,13 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>472881.36</v>
+        <v>422881.36</v>
       </c>
       <c r="G7" t="n">
-        <v>85118.64</v>
+        <v>76118.64</v>
       </c>
       <c r="H7" t="n">
-        <v>558000</v>
+        <v>499000</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -734,7 +734,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FA/31/2026</t>
+          <t>FN/45/2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>FA — Facture Avoir / Note de Crédit</t>
+          <t>FN — Facture Normale</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -758,13 +758,13 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>422881.36</v>
+        <v>8474.6</v>
       </c>
       <c r="G8" t="n">
-        <v>76118.64</v>
+        <v>1525.43</v>
       </c>
       <c r="H8" t="n">
-        <v>499000</v>
+        <v>10000.03</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -775,7 +775,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FN/45/2026</t>
+          <t>FN/46/2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -799,13 +799,13 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>8474.6</v>
+        <v>567796.64</v>
       </c>
       <c r="G9" t="n">
-        <v>1525.43</v>
+        <v>102203.4</v>
       </c>
       <c r="H9" t="n">
-        <v>10000.03</v>
+        <v>670000.04</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -816,7 +816,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FN/46/2026</t>
+          <t>FA/32/2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FN — Facture Normale</t>
+          <t>FA — Facture Avoir / Note de Crédit</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FA/32/2026</t>
+          <t>FN/47/2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>FA — Facture Avoir / Note de Crédit</t>
+          <t>FN — Facture Normale</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -881,13 +881,13 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>567796.64</v>
+        <v>109152.55</v>
       </c>
       <c r="G11" t="n">
-        <v>102203.4</v>
+        <v>19647.46</v>
       </c>
       <c r="H11" t="n">
-        <v>670000.04</v>
+        <v>128800.01</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -898,12 +898,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FN/47/2026</t>
+          <t>FN/43/2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -922,13 +922,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>109152.55</v>
+        <v>3389.84</v>
       </c>
       <c r="G12" t="n">
-        <v>19647.46</v>
+        <v>610.17</v>
       </c>
       <c r="H12" t="n">
-        <v>128800.01</v>
+        <v>4000.01</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FN/43/2026</t>
+          <t>FA/30/2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>FN — Facture Normale</t>
+          <t>FA — Facture Avoir / Note de Crédit</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -980,22 +980,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FA/30/2026</t>
+          <t>FN/41/2026</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ISM IRAKIZA SPARE MOTORS</t>
+          <t>Ndayishimiye emmanuel</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>FA — Facture Avoir / Note de Crédit</t>
+          <t>FN — Facture Normale</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1004,13 +1004,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>3389.84</v>
+        <v>378305.1</v>
       </c>
       <c r="G14" t="n">
-        <v>610.17</v>
+        <v>68094.91</v>
       </c>
       <c r="H14" t="n">
-        <v>4000.01</v>
+        <v>446400.01</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1021,7 +1021,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FN/41/2026</t>
+          <t>FN/42/2026</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1045,13 +1045,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>378305.1</v>
+        <v>102033.9</v>
       </c>
       <c r="G15" t="n">
-        <v>68094.91</v>
+        <v>18366.1</v>
       </c>
       <c r="H15" t="n">
-        <v>446400.01</v>
+        <v>120400</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1062,12 +1062,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FN/42/2026</t>
+          <t>FN/31/2026</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1086,13 +1086,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>102033.9</v>
+        <v>100000</v>
       </c>
       <c r="G16" t="n">
-        <v>18366.1</v>
+        <v>18000</v>
       </c>
       <c r="H16" t="n">
-        <v>120400</v>
+        <v>118000</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1103,7 +1103,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FN/31/2026</t>
+          <t>FA/21/2026</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>FN — Facture Normale</t>
+          <t>FA — Facture Avoir / Note de Crédit</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1144,7 +1144,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FA/21/2026</t>
+          <t>FA/22/2026</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1168,13 +1168,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>100000</v>
+        <v>200000</v>
       </c>
       <c r="G18" t="n">
-        <v>18000</v>
+        <v>36000</v>
       </c>
       <c r="H18" t="n">
-        <v>118000</v>
+        <v>236000</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1185,7 +1185,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FA/22/2026</t>
+          <t>FA/23/2026</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1226,7 +1226,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FA/23/2026</t>
+          <t>FA/24/2026</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1250,13 +1250,13 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>200000</v>
+        <v>3389.84</v>
       </c>
       <c r="G20" t="n">
-        <v>36000</v>
+        <v>610.17</v>
       </c>
       <c r="H20" t="n">
-        <v>236000</v>
+        <v>4000.01</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1267,7 +1267,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FA/24/2026</t>
+          <t>FA/25/2026</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1291,13 +1291,13 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3389.84</v>
+        <v>4067.8</v>
       </c>
       <c r="G21" t="n">
-        <v>610.17</v>
+        <v>732.2</v>
       </c>
       <c r="H21" t="n">
-        <v>4000.01</v>
+        <v>4800</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FA/25/2026</t>
+          <t>FA/26/2026</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1332,13 +1332,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>4067.8</v>
+        <v>372881.36</v>
       </c>
       <c r="G22" t="n">
-        <v>732.2</v>
+        <v>67118.64</v>
       </c>
       <c r="H22" t="n">
-        <v>4800</v>
+        <v>440000</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1349,7 +1349,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FA/26/2026</t>
+          <t>FA/27/2026</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1390,7 +1390,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FA/27/2026</t>
+          <t>FA/28/2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1414,13 +1414,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>372881.36</v>
+        <v>3389.84</v>
       </c>
       <c r="G24" t="n">
-        <v>67118.64</v>
+        <v>610.17</v>
       </c>
       <c r="H24" t="n">
-        <v>440000</v>
+        <v>4000.01</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1431,7 +1431,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>FA/28/2026</t>
+          <t>FN/32/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>FA — Facture Avoir / Note de Crédit</t>
+          <t>FN — Facture Normale</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1472,7 +1472,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FN/32/2026</t>
+          <t>FN/33/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1513,7 +1513,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>FN/33/2026</t>
+          <t>FN/34/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1537,13 +1537,13 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3389.84</v>
+        <v>372881.36</v>
       </c>
       <c r="G27" t="n">
-        <v>610.17</v>
+        <v>67118.64</v>
       </c>
       <c r="H27" t="n">
-        <v>4000.01</v>
+        <v>440000</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1554,7 +1554,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>FN/34/2026</t>
+          <t>FN/35/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1578,13 +1578,13 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>372881.36</v>
+        <v>100000</v>
       </c>
       <c r="G28" t="n">
-        <v>67118.64</v>
+        <v>18000</v>
       </c>
       <c r="H28" t="n">
-        <v>440000</v>
+        <v>118000</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1595,7 +1595,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>FN/35/2026</t>
+          <t>FN/36/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1619,13 +1619,13 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>100000</v>
+        <v>472881.36</v>
       </c>
       <c r="G29" t="n">
-        <v>18000</v>
+        <v>85118.64</v>
       </c>
       <c r="H29" t="n">
-        <v>118000</v>
+        <v>558000</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1636,7 +1636,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>FN/36/2026</t>
+          <t>FN/37/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1660,13 +1660,13 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>472881.36</v>
+        <v>8135.61</v>
       </c>
       <c r="G30" t="n">
-        <v>85118.64</v>
+        <v>1464.41</v>
       </c>
       <c r="H30" t="n">
-        <v>558000</v>
+        <v>9600.02</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -1677,7 +1677,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>FN/37/2026</t>
+          <t>FN/38/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1701,13 +1701,13 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>8135.61</v>
+        <v>378305.1</v>
       </c>
       <c r="G31" t="n">
-        <v>1464.41</v>
+        <v>68094.91</v>
       </c>
       <c r="H31" t="n">
-        <v>9600.02</v>
+        <v>446400.01</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -1718,7 +1718,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>FN/38/2026</t>
+          <t>FN/39/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1742,13 +1742,13 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>378305.1</v>
+        <v>239152.55</v>
       </c>
       <c r="G32" t="n">
-        <v>68094.91</v>
+        <v>43047.46</v>
       </c>
       <c r="H32" t="n">
-        <v>446400.01</v>
+        <v>282200.01</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -1759,7 +1759,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>FN/39/2026</t>
+          <t>FA/29/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>FN — Facture Normale</t>
+          <t>FA — Facture Avoir / Note de Crédit</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1800,7 +1800,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>FA/29/2026</t>
+          <t>FN/40/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>FA — Facture Avoir / Note de Crédit</t>
+          <t>FN — Facture Normale</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1824,13 +1824,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>239152.55</v>
+        <v>2711.87</v>
       </c>
       <c r="G34" t="n">
-        <v>43047.46</v>
+        <v>488.14</v>
       </c>
       <c r="H34" t="n">
-        <v>282200.01</v>
+        <v>3200.01</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -1841,12 +1841,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>FN/40/2026</t>
+          <t>FN/20/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>03/04/2026</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1865,13 +1865,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2711.87</v>
+        <v>3389.84</v>
       </c>
       <c r="G35" t="n">
-        <v>488.14</v>
+        <v>610.17</v>
       </c>
       <c r="H35" t="n">
-        <v>3200.01</v>
+        <v>4000.01</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -1882,7 +1882,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>FN/20/2026</t>
+          <t>FN/21/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1906,13 +1906,13 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3389.84</v>
+        <v>372881.36</v>
       </c>
       <c r="G36" t="n">
-        <v>610.17</v>
+        <v>67118.64</v>
       </c>
       <c r="H36" t="n">
-        <v>4000.01</v>
+        <v>440000</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>FN/21/2026</t>
+          <t>FN/22/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1947,13 +1947,13 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>372881.36</v>
+        <v>2033.9</v>
       </c>
       <c r="G37" t="n">
-        <v>67118.64</v>
+        <v>366.1</v>
       </c>
       <c r="H37" t="n">
-        <v>440000</v>
+        <v>2400</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -1964,7 +1964,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>FN/22/2026</t>
+          <t>FN/23/2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2005,7 +2005,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>FN/23/2026</t>
+          <t>FA/20/2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>FN — Facture Normale</t>
+          <t>FA — Facture Avoir / Note de Crédit</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2029,13 +2029,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>2033.9</v>
+        <v>3389.84</v>
       </c>
       <c r="G39" t="n">
-        <v>366.1</v>
+        <v>610.17</v>
       </c>
       <c r="H39" t="n">
-        <v>2400</v>
+        <v>4000.01</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -2046,7 +2046,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>FA/20/2026</t>
+          <t>FN/24/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>FA — Facture Avoir / Note de Crédit</t>
+          <t>FN — Facture Normale</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2070,13 +2070,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3389.84</v>
+        <v>372881.36</v>
       </c>
       <c r="G40" t="n">
-        <v>610.17</v>
+        <v>67118.64</v>
       </c>
       <c r="H40" t="n">
-        <v>4000.01</v>
+        <v>440000</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -2087,7 +2087,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>FN/24/2026</t>
+          <t>FN/25/2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2111,13 +2111,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>372881.36</v>
+        <v>3389.84</v>
       </c>
       <c r="G41" t="n">
-        <v>67118.64</v>
+        <v>610.17</v>
       </c>
       <c r="H41" t="n">
-        <v>440000</v>
+        <v>4000.01</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>FN/25/2026</t>
+          <t>FN/26/2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2152,13 +2152,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3389.84</v>
+        <v>1694.92</v>
       </c>
       <c r="G42" t="n">
-        <v>610.17</v>
+        <v>305.09</v>
       </c>
       <c r="H42" t="n">
-        <v>4000.01</v>
+        <v>2000.01</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -2169,7 +2169,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>FN/26/2026</t>
+          <t>FN/27/2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2193,13 +2193,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>1694.92</v>
+        <v>372881.36</v>
       </c>
       <c r="G43" t="n">
-        <v>305.09</v>
+        <v>67118.64</v>
       </c>
       <c r="H43" t="n">
-        <v>2000.01</v>
+        <v>440000</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
@@ -2210,7 +2210,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>FN/27/2026</t>
+          <t>FN/28/2026</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2234,13 +2234,13 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>372881.36</v>
+        <v>4067.8</v>
       </c>
       <c r="G44" t="n">
-        <v>67118.64</v>
+        <v>732.2</v>
       </c>
       <c r="H44" t="n">
-        <v>440000</v>
+        <v>4800</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -2251,7 +2251,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>FN/28/2026</t>
+          <t>FN/29/2026</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2275,13 +2275,13 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>4067.8</v>
+        <v>50000</v>
       </c>
       <c r="G45" t="n">
-        <v>732.2</v>
+        <v>9000</v>
       </c>
       <c r="H45" t="n">
-        <v>4800</v>
+        <v>59000</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2292,7 +2292,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>FN/29/2026</t>
+          <t>FN/30/2026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2316,56 +2316,15 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>50000</v>
+        <v>200000</v>
       </c>
       <c r="G46" t="n">
-        <v>9000</v>
+        <v>36000</v>
       </c>
       <c r="H46" t="n">
-        <v>59000</v>
+        <v>236000</v>
       </c>
       <c r="I46" t="inlineStr">
-        <is>
-          <t>ENVOYE</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>FN/30/2026</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>03/04/2026</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Ndayishimiye emmanuel</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>FN — Facture Normale</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F47" t="n">
-        <v>200000</v>
-      </c>
-      <c r="G47" t="n">
-        <v>36000</v>
-      </c>
-      <c r="H47" t="n">
-        <v>236000</v>
-      </c>
-      <c r="I47" t="inlineStr">
         <is>
           <t>ENVOYE</t>
         </is>

</xml_diff>